<commit_message>
fix: clean startup — resolve prisma client model name mismatches, add ATL/BTL split, signal layer
</commit_message>
<xml_diff>
--- a/tests/sample_data/Echoes_2026-06-07.csv.xlsx
+++ b/tests/sample_data/Echoes_2026-06-07.csv.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\SceneIQ-Compliance\tests\sample_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{47583CA1-1B55-4D6B-BCD7-E0661B263EB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A3E28C53-0AB9-49E4-8AB3-18F08835EDF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{14AC49B3-8E57-48CC-BA41-95FEDDE5B97C}"/>
   </bookViews>
   <sheets>
     <sheet name="Echoes_2026-06-07" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="0" iterateDelta="1E-4"/>
+  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
@@ -992,7 +993,11 @@
   <dimension ref="A1:F11"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
+    <col min="1" max="1" width="28.6328125" customWidth="1"/>
+    <col min="2" max="2" width="41.7265625" customWidth="1"/>
     <col min="3" max="3" width="27.453125" customWidth="1"/>
+    <col min="4" max="4" width="39.26953125" customWidth="1"/>
+    <col min="5" max="5" width="32.08984375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">

</xml_diff>